<commit_message>
feat: update candidate facts to Expected CTC 10 LPA, Immediate Joiner, add UI External/Failed tabs and Gmail OTP helper
</commit_message>
<xml_diff>
--- a/backend/data/job-applications.xlsx
+++ b/backend/data/job-applications.xlsx
@@ -828,7 +828,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I333"/>
+  <dimension ref="A1:I353"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -10498,9 +10498,589 @@
         <v>External — apply manually</v>
       </c>
     </row>
+    <row r="334">
+      <c r="A334">
+        <v>333</v>
+      </c>
+      <c r="B334" t="str">
+        <v>2/9/2026, 12:49:56 pm</v>
+      </c>
+      <c r="C334" t="str">
+        <v>naukri_external</v>
+      </c>
+      <c r="D334" t="str">
+        <v>Custom Software Engineer</v>
+      </c>
+      <c r="E334" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F334" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G334" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-310826920170</v>
+      </c>
+      <c r="H334" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-310826920170</v>
+      </c>
+      <c r="I334" t="str">
+        <v>Captured form state (0 fields)</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335">
+        <v>334</v>
+      </c>
+      <c r="B335" t="str">
+        <v>2/9/2026, 12:50:01 pm</v>
+      </c>
+      <c r="C335" t="str">
+        <v>naukri_external</v>
+      </c>
+      <c r="D335" t="str">
+        <v>Application Developer</v>
+      </c>
+      <c r="E335" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F335" t="str">
+        <v>Hyderabad, Mumbai</v>
+      </c>
+      <c r="G335" t="str">
+        <v>https://www.naukri.com/job-listings-application-developer-accenture-solutions-pvt-ltd-mumbai-hyderabad-2-to-5-years-170826921174</v>
+      </c>
+      <c r="H335" t="str">
+        <v>https://www.naukri.com/job-listings-application-developer-accenture-solutions-pvt-ltd-mumbai-hyderabad-2-to-5-years-170826921174</v>
+      </c>
+      <c r="I335" t="str">
+        <v>Captured form state (0 fields)</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336">
+        <v>335</v>
+      </c>
+      <c r="B336" t="str">
+        <v>2/9/2026, 12:50:06 pm</v>
+      </c>
+      <c r="C336" t="str">
+        <v>naukri_external</v>
+      </c>
+      <c r="D336" t="str">
+        <v>Software Development Engineer</v>
+      </c>
+      <c r="E336" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F336" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G336" t="str">
+        <v>https://www.naukri.com/job-listings-software-development-engineer-accenture-solutions-pvt-ltd-hyderabad-1-to-4-years-170826923848</v>
+      </c>
+      <c r="H336" t="str">
+        <v>https://www.naukri.com/job-listings-software-development-engineer-accenture-solutions-pvt-ltd-hyderabad-1-to-4-years-170826923848</v>
+      </c>
+      <c r="I336" t="str">
+        <v>Captured form state (0 fields)</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337">
+        <v>336</v>
+      </c>
+      <c r="B337" t="str">
+        <v>2/9/2026, 12:50:10 pm</v>
+      </c>
+      <c r="C337" t="str">
+        <v>naukri_external</v>
+      </c>
+      <c r="D337" t="str">
+        <v>Application Developer</v>
+      </c>
+      <c r="E337" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F337" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G337" t="str">
+        <v>https://www.naukri.com/job-listings-application-developer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-310826918711</v>
+      </c>
+      <c r="H337" t="str">
+        <v>https://www.naukri.com/job-listings-application-developer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-310826918711</v>
+      </c>
+      <c r="I337" t="str">
+        <v>Captured form state (0 fields)</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338">
+        <v>337</v>
+      </c>
+      <c r="B338" t="str">
+        <v>2/9/2026, 12:50:15 pm</v>
+      </c>
+      <c r="C338" t="str">
+        <v>naukri_external</v>
+      </c>
+      <c r="D338" t="str">
+        <v>Application Developer</v>
+      </c>
+      <c r="E338" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F338" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G338" t="str">
+        <v>https://www.naukri.com/job-listings-application-developer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-310826917881</v>
+      </c>
+      <c r="H338" t="str">
+        <v>https://www.naukri.com/job-listings-application-developer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-310826917881</v>
+      </c>
+      <c r="I338" t="str">
+        <v>Captured form state (0 fields)</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339">
+        <v>338</v>
+      </c>
+      <c r="B339" t="str">
+        <v>2/9/2026, 12:50:19 pm</v>
+      </c>
+      <c r="C339" t="str">
+        <v>naukri_external</v>
+      </c>
+      <c r="D339" t="str">
+        <v>Application Developer</v>
+      </c>
+      <c r="E339" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F339" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G339" t="str">
+        <v>https://www.naukri.com/job-listings-application-developer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-010926932687</v>
+      </c>
+      <c r="H339" t="str">
+        <v>https://www.naukri.com/job-listings-application-developer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-010926932687</v>
+      </c>
+      <c r="I339" t="str">
+        <v>Captured form state (0 fields)</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340">
+        <v>339</v>
+      </c>
+      <c r="B340" t="str">
+        <v>2/9/2026, 12:50:24 pm</v>
+      </c>
+      <c r="C340" t="str">
+        <v>naukri_external</v>
+      </c>
+      <c r="D340" t="str">
+        <v>Java Developer Spring Boot Flink &amp; Kafka</v>
+      </c>
+      <c r="E340" t="str">
+        <v>Stellar Technologies</v>
+      </c>
+      <c r="F340" t="str">
+        <v>Hyderabad, Mumbai, Kolkata, New Delhi, Pune, Chennai, Bengaluru</v>
+      </c>
+      <c r="G340" t="str">
+        <v>https://www.naukri.com/job-listings-java-developer-spring-boot-flink-kafka-stellar-technologies-kolkata-mumbai-new-delhi-hyderabad-pune-chennai-bengaluru-2-to-4-years-220525505217</v>
+      </c>
+      <c r="H340" t="str">
+        <v>https://www.naukri.com/job-listings-java-developer-spring-boot-flink-kafka-stellar-technologies-kolkata-mumbai-new-delhi-hyderabad-pune-chennai-bengaluru-2-to-4-years-220525505217</v>
+      </c>
+      <c r="I340" t="str">
+        <v>Captured form state (0 fields)</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341">
+        <v>340</v>
+      </c>
+      <c r="B341" t="str">
+        <v>2/9/2026, 12:50:28 pm</v>
+      </c>
+      <c r="C341" t="str">
+        <v>naukri_external</v>
+      </c>
+      <c r="D341" t="str">
+        <v>Custom Software Engineer</v>
+      </c>
+      <c r="E341" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F341" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G341" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-3-to-5-years-310826918541</v>
+      </c>
+      <c r="H341" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-3-to-5-years-310826918541</v>
+      </c>
+      <c r="I341" t="str">
+        <v>Captured form state (0 fields)</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342">
+        <v>341</v>
+      </c>
+      <c r="B342" t="str">
+        <v>2/9/2026, 12:50:33 pm</v>
+      </c>
+      <c r="C342" t="str">
+        <v>naukri_external</v>
+      </c>
+      <c r="D342" t="str">
+        <v>Application Developer-Cloud FullStack</v>
+      </c>
+      <c r="E342" t="str">
+        <v>IBM</v>
+      </c>
+      <c r="F342" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G342" t="str">
+        <v>https://www.naukri.com/job-listings-application-developer-cloud-fullstack-ibm-india-pvt-limited-hyderabad-3-to-8-years-260826923637</v>
+      </c>
+      <c r="H342" t="str">
+        <v>https://www.naukri.com/job-listings-application-developer-cloud-fullstack-ibm-india-pvt-limited-hyderabad-3-to-8-years-260826923637</v>
+      </c>
+      <c r="I342" t="str">
+        <v>Captured form state (0 fields)</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343">
+        <v>342</v>
+      </c>
+      <c r="B343" t="str">
+        <v>2/9/2026, 12:50:38 pm</v>
+      </c>
+      <c r="C343" t="str">
+        <v>naukri_external</v>
+      </c>
+      <c r="D343" t="str">
+        <v>Full Stack Developer - Java</v>
+      </c>
+      <c r="E343" t="str">
+        <v>Proounce</v>
+      </c>
+      <c r="F343" t="str">
+        <v>Hyderabad, Mumbai, Kolkata, New Delhi, Pune, Chennai, Bengaluru</v>
+      </c>
+      <c r="G343" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-java-proounce-solutions-private-limited-kolkata-mumbai-new-delhi-hyderabad-pune-chennai-bengaluru-6-to-10-years-141024501812</v>
+      </c>
+      <c r="H343" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-java-proounce-solutions-private-limited-kolkata-mumbai-new-delhi-hyderabad-pune-chennai-bengaluru-6-to-10-years-141024501812</v>
+      </c>
+      <c r="I343" t="str">
+        <v>Captured form state (0 fields)</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344">
+        <v>343</v>
+      </c>
+      <c r="B344" t="str">
+        <v>2/9/2026, 12:50:42 pm</v>
+      </c>
+      <c r="C344" t="str">
+        <v>naukri_external</v>
+      </c>
+      <c r="D344" t="str">
+        <v>Full Stack Developer - Project Alpha</v>
+      </c>
+      <c r="E344" t="str">
+        <v>Avataa Solutions</v>
+      </c>
+      <c r="F344" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G344" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-project-alpha-avataa-solutions-hyderabad-3-to-7-years-150526502877</v>
+      </c>
+      <c r="H344" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-project-alpha-avataa-solutions-hyderabad-3-to-7-years-150526502877</v>
+      </c>
+      <c r="I344" t="str">
+        <v>Captured form state (0 fields)</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345">
+        <v>344</v>
+      </c>
+      <c r="B345" t="str">
+        <v>2/9/2026, 12:50:47 pm</v>
+      </c>
+      <c r="C345" t="str">
+        <v>naukri_external</v>
+      </c>
+      <c r="D345" t="str">
+        <v>AI Augmented Full Stack Engineer</v>
+      </c>
+      <c r="E345" t="str">
+        <v>I5 Systems</v>
+      </c>
+      <c r="F345" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G345" t="str">
+        <v>https://www.naukri.com/job-listings-ai-augmented-full-stack-engineer-i5-systems-hyderabad-3-to-7-years-010526502998</v>
+      </c>
+      <c r="H345" t="str">
+        <v>https://www.naukri.com/job-listings-ai-augmented-full-stack-engineer-i5-systems-hyderabad-3-to-7-years-010526502998</v>
+      </c>
+      <c r="I345" t="str">
+        <v>Captured form state (0 fields)</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346">
+        <v>345</v>
+      </c>
+      <c r="B346" t="str">
+        <v>2/9/2026, 12:50:51 pm</v>
+      </c>
+      <c r="C346" t="str">
+        <v>naukri_external</v>
+      </c>
+      <c r="D346" t="str">
+        <v>Custom Software Engineer</v>
+      </c>
+      <c r="E346" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F346" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G346" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-3-to-8-years-240826926095</v>
+      </c>
+      <c r="H346" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-3-to-8-years-240826926095</v>
+      </c>
+      <c r="I346" t="str">
+        <v>Captured form state (0 fields)</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347">
+        <v>346</v>
+      </c>
+      <c r="B347" t="str">
+        <v>2/9/2026, 12:50:56 pm</v>
+      </c>
+      <c r="C347" t="str">
+        <v>naukri_external</v>
+      </c>
+      <c r="D347" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E347" t="str">
+        <v>Annnetwork</v>
+      </c>
+      <c r="F347" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G347" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-annnetwork-hyderabad-3-to-5-years-121125501120</v>
+      </c>
+      <c r="H347" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-annnetwork-hyderabad-3-to-5-years-121125501120</v>
+      </c>
+      <c r="I347" t="str">
+        <v>Captured form state (0 fields)</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348">
+        <v>347</v>
+      </c>
+      <c r="B348" t="str">
+        <v>2/9/2026, 12:51:00 pm</v>
+      </c>
+      <c r="C348" t="str">
+        <v>naukri_external</v>
+      </c>
+      <c r="D348" t="str">
+        <v>Custom Software Engineer</v>
+      </c>
+      <c r="E348" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F348" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G348" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-110826934178</v>
+      </c>
+      <c r="H348" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-110826934178</v>
+      </c>
+      <c r="I348" t="str">
+        <v>Captured form state (0 fields)</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349">
+        <v>348</v>
+      </c>
+      <c r="B349" t="str">
+        <v>2/9/2026, 12:51:05 pm</v>
+      </c>
+      <c r="C349" t="str">
+        <v>naukri_external</v>
+      </c>
+      <c r="D349" t="str">
+        <v>Java + React Full Stack Developer</v>
+      </c>
+      <c r="E349" t="str">
+        <v>Orbion Infotech</v>
+      </c>
+      <c r="F349" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G349" t="str">
+        <v>https://www.naukri.com/job-listings-java-react-full-stack-developer-orbion-infotech-hyderabad-7-to-8-years-010926503869</v>
+      </c>
+      <c r="H349" t="str">
+        <v>https://www.naukri.com/job-listings-java-react-full-stack-developer-orbion-infotech-hyderabad-7-to-8-years-010926503869</v>
+      </c>
+      <c r="I349" t="str">
+        <v>Captured form state (0 fields)</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350">
+        <v>349</v>
+      </c>
+      <c r="B350" t="str">
+        <v>2/9/2026, 12:51:10 pm</v>
+      </c>
+      <c r="C350" t="str">
+        <v>naukri_external</v>
+      </c>
+      <c r="D350" t="str">
+        <v>Application Developer</v>
+      </c>
+      <c r="E350" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F350" t="str">
+        <v>Hyderabad, Mumbai</v>
+      </c>
+      <c r="G350" t="str">
+        <v>https://www.naukri.com/job-listings-application-developer-accenture-solutions-pvt-ltd-mumbai-hyderabad-3-to-8-years-110826931532</v>
+      </c>
+      <c r="H350" t="str">
+        <v>https://www.naukri.com/job-listings-application-developer-accenture-solutions-pvt-ltd-mumbai-hyderabad-3-to-8-years-110826931532</v>
+      </c>
+      <c r="I350" t="str">
+        <v>Captured form state (0 fields)</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351">
+        <v>350</v>
+      </c>
+      <c r="B351" t="str">
+        <v>2/9/2026, 12:51:14 pm</v>
+      </c>
+      <c r="C351" t="str">
+        <v>naukri_external</v>
+      </c>
+      <c r="D351" t="str">
+        <v>Application Developer</v>
+      </c>
+      <c r="E351" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F351" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G351" t="str">
+        <v>https://www.naukri.com/job-listings-application-developer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-170826925605</v>
+      </c>
+      <c r="H351" t="str">
+        <v>https://www.naukri.com/job-listings-application-developer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-170826925605</v>
+      </c>
+      <c r="I351" t="str">
+        <v>Captured form state (0 fields)</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352">
+        <v>351</v>
+      </c>
+      <c r="B352" t="str">
+        <v>2/9/2026, 12:51:19 pm</v>
+      </c>
+      <c r="C352" t="str">
+        <v>naukri_external</v>
+      </c>
+      <c r="D352" t="str">
+        <v>Application Developer</v>
+      </c>
+      <c r="E352" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F352" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G352" t="str">
+        <v>https://www.naukri.com/job-listings-application-developer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-170826924949</v>
+      </c>
+      <c r="H352" t="str">
+        <v>https://www.naukri.com/job-listings-application-developer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-170826924949</v>
+      </c>
+      <c r="I352" t="str">
+        <v>Captured form state (0 fields)</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353">
+        <v>352</v>
+      </c>
+      <c r="B353" t="str">
+        <v>2/9/2026, 12:51:23 pm</v>
+      </c>
+      <c r="C353" t="str">
+        <v>naukri_external</v>
+      </c>
+      <c r="D353" t="str">
+        <v>Application Developer</v>
+      </c>
+      <c r="E353" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F353" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G353" t="str">
+        <v>https://www.naukri.com/job-listings-application-developer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-310826918599</v>
+      </c>
+      <c r="H353" t="str">
+        <v>https://www.naukri.com/job-listings-application-developer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-310826918599</v>
+      </c>
+      <c r="I353" t="str">
+        <v>Captured form state (0 fields)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I333"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I353"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: transform UI into pure Job Application Tracker dashboard with manual CLI & UI logger
</commit_message>
<xml_diff>
--- a/backend/data/job-applications.xlsx
+++ b/backend/data/job-applications.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I15"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -819,9 +819,38 @@
         <v>Naukri quick-apply (auto)</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>2/9/2026, 5:12:38 pm</v>
+      </c>
+      <c r="C15" t="str">
+        <v>manual_external</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Google</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G15" t="str">
+        <v>https://careers.google.com/jobs/123</v>
+      </c>
+      <c r="H15" t="str">
+        <v>https://careers.google.com/jobs/123</v>
+      </c>
+      <c r="I15" t="str">
+        <v>Applied via Google Careers</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I15"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>